<commit_message>
Added financials for 2021
</commit_message>
<xml_diff>
--- a/excel/MSFT_DCF_Model.xlsx
+++ b/excel/MSFT_DCF_Model.xlsx
@@ -569,43 +569,43 @@
         <v>2021</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v/>
+        <v>168088000000</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v/>
+        <v>115856000000</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v/>
+        <v>69916000000</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v/>
+        <v>61271000000</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v/>
+        <v>0.689258007710247</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v/>
+        <v>0.415948788729713</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v/>
+        <v>0.138266152850834</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v/>
+        <v>11689000000</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v/>
+        <v>20622000000</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v/>
+        <v>56118000000</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v/>
+        <v>67775000000</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v/>
+        <v>14224000000</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v/>
+        <v>95749000000</v>
       </c>
     </row>
     <row r="6">
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3166936236032</v>
+        <v>3152517529600</v>
       </c>
     </row>
     <row r="8">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>426.1</v>
+        <v>424.16</v>
       </c>
     </row>
     <row r="9">

</xml_diff>